<commit_message>
feat: verify rule CG0297 and add negative test cases
</commit_message>
<xml_diff>
--- a/rules/CORE-000157/negative/01/data/unit-test-coreid-CG0297-negative.xlsx
+++ b/rules/CORE-000157/negative/01/data/unit-test-coreid-CG0297-negative.xlsx
@@ -35,7 +35,7 @@
       <i val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -46,6 +46,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFCC"/>
         <bgColor rgb="00FFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -76,7 +82,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -86,6 +92,9 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -529,7 +538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -561,6 +570,34 @@
       <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Error value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>tv.xpt</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>7</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ARMCD</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>AA-BB-AA-BB-AA-BB-AAA</t>
         </is>
       </c>
     </row>
@@ -825,7 +862,7 @@
       <c r="E7" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>AA-BB-AA-BB-AA-BB-AAA</t>
         </is>

</xml_diff>